<commit_message>
Add guided AI preparation prompt to import workbook
</commit_message>
<xml_diff>
--- a/assets/import/Pico-import.xlsx
+++ b/assets/import/Pico-import.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +72,82 @@
       <color rgb="001A2151"/>
       <sz val="16"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1A2151"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF8A92A8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF9A8540"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF1F7AEA"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F7AEA"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1A2151"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1A2151"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1A2151"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF1F7AEA"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF6B7389"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -90,8 +164,29 @@
         <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F6FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F6FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -129,11 +224,64 @@
         <color rgb="00E3E7EE"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFE3E7EE"/>
+      </right>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFE3E7EE"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FFC9D2E0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE3E7EE"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFE3E7EE"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FFE3E7EE"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDCE8FA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDCE8FA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDCE8FA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDCE8FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,6 +318,66 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="1"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" xfId="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" xfId="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="7" borderId="9" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="7" borderId="9" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="7" borderId="9" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="9" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="1"/>
+    <xf numFmtId="1" fontId="13" fillId="4" borderId="9" xfId="1"/>
+    <xf numFmtId="1" fontId="15" fillId="4" borderId="9" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,92 +741,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="140" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="140" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
-          <t>Как заполнять</t>
+          <t xml:space="preserve">Как заполнять</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="39" t="str">
+        <v>Перенесите данные из своих файлов с помощью ИИ</v>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="B4" s="38" t="str">
+        <v>1. Приложите этот шаблон и свои старые или незаполненные до конца Excel-файлы к сообщению помощнику. Для Google Docs дайте доступную ему ссылку или приложите экспорт документа.</v>
+      </c>
+    </row>
+    <row r="5" ht="23" customHeight="1">
+      <c r="B5" s="38" t="str">
+        <v>2. Скопируйте готовый запрос ниже и отправьте его вместе с файлами.</v>
+      </c>
+    </row>
+    <row r="6" ht="23" customHeight="1">
+      <c r="B6" s="40" t="str">
+        <v>Передавайте внешнему помощнику только те данные, которыми разрешено делиться.</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="38"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="B8" s="39" t="str">
+        <v>Готовый запрос — скопируйте текст из ячейки ниже</v>
+      </c>
+    </row>
+    <row r="9" ht="215" customHeight="1">
+      <c r="B9" s="43" t="str">
+        <v>Перенеси сведения из приложенных файлов и доступных Google Docs в шаблон Pico-import.xlsx. Верни заполненный файл XLSX.
+Сохрани три листа, их названия и порядок, заголовки, колонки, оформление и формулы. Предзаполненные примеры сохрани как примеры, не считай их моими данными. Новые данные размещай ниже примера: одна строка — одна компания или один проект. Свяжи проекты с компаниями по названию и ИНН.
+Используй только сведения из источников. Не придумывай ИНН, даты, стадии или потенциал. Неизвестные поля оставляй пустыми; пустые суммы не заменяй нулями. Суммы в шаблоне — в млн ₽: пересчитывай их только при явно известных исходных единицах.
+Все контакты компании запиши в одну ячейку «Контакты», каждый с новой строки внутри ячейки: ФИО, должность, телефон, email. Для пропущенного поля сохраняй запятые. Не дублируй строку компании ради контактов.
+Если сведения противоречат друг другу, непонятно, к какой компании относится проект, или неизвестны единицы суммы — сначала задай вопросы. Если ссылка недоступна, попроси файл или экспорт документа. Не теряй сведения молча.
+Верни заполненный XLSX и кратко перечисли вопросы и сведения, которые не удалось перенести.</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="38"/>
+    </row>
+    <row r="11" ht="35" customHeight="1">
+      <c r="B11" s="38" t="str">
+        <v>3. Проверьте полученный Excel и отправьте его в чат Pico. Бот покажет предпросмотр и сохранит данные только после вашего подтверждения.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="38"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="39" t="str">
+        <v>Правила заполнения</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>1.  Два листа: «Клиенты» (кто это) и «Проекты» (что у них в работе). Жёлтая строка - пример, своё пишите ниже.</t>
+          <t xml:space="preserve">1.  Два листа: «Клиенты» (кто это) и «Проекты» (что у них в работе). Жёлтая строка - пример, своё пишите ниже.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>2.  Клиенты: одна строка - один клиент. Обязательно: ИНН, Компания, Тип клиента. Остальное - что знаете.</t>
+          <t xml:space="preserve">2.  Клиенты: одна строка - один клиент. Обязательно: ИНН, Компания, Тип клиента. Остальное - что знаете.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="2" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>3.  Проекты: одна строка - один проект. В первых двух колонках - компания, которая принесла проект, и её ИНН. Затем заказчик проекта и его ИНН.</t>
+          <t xml:space="preserve">3.  Проекты: одна строка - один проект. В первых двух колонках - компания, которая принесла проект, и её ИНН. Затем заказчик проекта и его ИНН.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="2" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>4.  Где написано «из списка» - нажмите на ячейку и выберите вариант стрелкой справа.</t>
+          <t xml:space="preserve">4.  Где написано «из списка» - нажмите на ячейку и выберите вариант стрелкой справа.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="2" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>5.  Компания и заказчик - только название: Щит-Энерго, без ООО и кавычек. Якорные заказчики - так же, несколько через запятую.</t>
+          <t xml:space="preserve">5.  Компания и заказчик - только название: Щит-Энерго, без ООО и кавычек. Якорные заказчики - так же, несколько через запятую.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="2" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>6.  Суммы - в млн ₽, без запятой (округлите), в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
+          <t xml:space="preserve">6.  Суммы - в млн ₽, без запятой (округлите), в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>7.  Контакты: в одной ячейке, как в примере - ФИО, должность, телефон, почта. Следующий контакт - с новой строки в той же ячейке (Windows: Alt+Enter, Mac: Ctrl+Option+Enter).</t>
+          <t xml:space="preserve">7.  Контакты: в одной ячейке, как в примере - ФИО, должность, телефон, почта. Следующий контакт - с новой строки в той же ячейке (Windows: Alt+Enter, Mac: Ctrl+Option+Enter).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>8.  Оборудование, которого нет в колонках, пишите в «Другое»: название, тире, сумма. Например: Трансформатор - 2.</t>
+          <t xml:space="preserve">8.  Оборудование, которого нет в колонках, пишите в «Другое»: название, тире, сумма. Например: Трансформатор - 2.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="2" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>9.  Даты - месяц и год, например 03.2027. Комментарий - пара коротких тезисов.</t>
+          <t xml:space="preserve">9.  Даты - месяц и год, например 03.2027. Комментарий - пара коротких тезисов.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add inline client workflows, holding relationships and import normalization
</commit_message>
<xml_diff>
--- a/assets/import/Pico-import.xlsx
+++ b/assets/import/Pico-import.xlsx
@@ -825,7 +825,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.  Клиенты: одна строка - один клиент. Обязательно: ИНН, Компания, Тип клиента. Остальное - что знаете.</t>
+          <t xml:space="preserve">2.  Клиенты: одна строка - один клиент. Обязательно: Компания и Тип клиента; ИНН обязателен, кроме холдингов. Остальное - что знаете.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.  Суммы - в млн ₽, без запятой (округлите), в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
+          <t xml:space="preserve">6.  Суммы - в млн ₽, можно с дробной частью, в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11670,7 @@
   </mergeCells>
   <dataValidations count="7">
     <dataValidation sqref="A4:A504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="ИНН" error="ИНН - 10 или 12 цифр, без пробелов и букв" promptTitle="ИНН" prompt="Только цифры: 10 у компании, 12 у ИП" type="custom">
-      <formula1>=AND(ISNUMBER(--A4),OR(LEN(A4)=10,LEN(A4)=12))</formula1>
+      <formula1>=OR(AND(D4="Холдинг",A4=""),AND(D4&lt;&gt;"Холдинг",ISNUMBER(--A4),OR(LEN(A4)=10,LEN(A4)=12)))</formula1>
     </dataValidation>
     <dataValidation sqref="B4:B504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Компания" error="Уберите ООО/АО/ИП и кавычки - только название" promptTitle="Компания" prompt="Только название: Щит-Энерго, а не ООО «Щит-Энерго»" type="custom">
       <formula1>=AND(ISERROR(SEARCH("""",B4)),ISERROR(SEARCH("«",B4)),ISERROR(SEARCH("»",B4)),LEFT(B4,4)&lt;&gt;"ООО ",LEFT(B4,3)&lt;&gt;"АО ",LEFT(B4,4)&lt;&gt;"ПАО ",LEFT(B4,4)&lt;&gt;"ЗАО ",LEFT(B4,4)&lt;&gt;"ОАО ",LEFT(B4,3)&lt;&gt;"ИП ",LEN(B4)&lt;=40)</formula1>
@@ -11679,7 +11679,7 @@
       <formula1>30</formula1>
     </dataValidation>
     <dataValidation sqref="D4:D504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Тип клиента" error="Выберите вариант из списка" promptTitle="Тип клиента" prompt="Выберите один вариант" type="list">
-      <formula1>"Заказчик,Подрядчик,Сетевая компания,Проектный институт,Интегратор,Коммерческая организация,OEM"</formula1>
+      <formula1>"Холдинг,Заказчик,Подрядчик,Интегратор,Сетевая компания,OEM,Дистрибьютор,Проектный институт"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:L504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Потенциал" error="Только целое число, без запятой: 5, а не 5,5" promptTitle="Потенциал" prompt="Сумма в млн ₽ в год, без запятой. Нет потенциала - оставьте пустым" type="whole" operator="between">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Add inline client workflows, holding relationships and import normalization (#17)
Co-authored-by: v.savin <szt-vadim@yandex.ru>
</commit_message>
<xml_diff>
--- a/assets/import/Pico-import.xlsx
+++ b/assets/import/Pico-import.xlsx
@@ -825,7 +825,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.  Клиенты: одна строка - один клиент. Обязательно: ИНН, Компания, Тип клиента. Остальное - что знаете.</t>
+          <t xml:space="preserve">2.  Клиенты: одна строка - один клиент. Обязательно: Компания и Тип клиента; ИНН обязателен, кроме холдингов. Остальное - что знаете.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.  Суммы - в млн ₽, без запятой (округлите), в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
+          <t xml:space="preserve">6.  Суммы - в млн ₽, можно с дробной частью, в нужную колонку. Выключатели и ПЧ (УПП) делятся на 0,4 кВ и 6-35 кВ. Нет суммы - оставьте пустым.</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11670,7 @@
   </mergeCells>
   <dataValidations count="7">
     <dataValidation sqref="A4:A504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="ИНН" error="ИНН - 10 или 12 цифр, без пробелов и букв" promptTitle="ИНН" prompt="Только цифры: 10 у компании, 12 у ИП" type="custom">
-      <formula1>=AND(ISNUMBER(--A4),OR(LEN(A4)=10,LEN(A4)=12))</formula1>
+      <formula1>=OR(AND(D4="Холдинг",A4=""),AND(D4&lt;&gt;"Холдинг",ISNUMBER(--A4),OR(LEN(A4)=10,LEN(A4)=12)))</formula1>
     </dataValidation>
     <dataValidation sqref="B4:B504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Компания" error="Уберите ООО/АО/ИП и кавычки - только название" promptTitle="Компания" prompt="Только название: Щит-Энерго, а не ООО «Щит-Энерго»" type="custom">
       <formula1>=AND(ISERROR(SEARCH("""",B4)),ISERROR(SEARCH("«",B4)),ISERROR(SEARCH("»",B4)),LEFT(B4,4)&lt;&gt;"ООО ",LEFT(B4,3)&lt;&gt;"АО ",LEFT(B4,4)&lt;&gt;"ПАО ",LEFT(B4,4)&lt;&gt;"ЗАО ",LEFT(B4,4)&lt;&gt;"ОАО ",LEFT(B4,3)&lt;&gt;"ИП ",LEN(B4)&lt;=40)</formula1>
@@ -11679,7 +11679,7 @@
       <formula1>30</formula1>
     </dataValidation>
     <dataValidation sqref="D4:D504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Тип клиента" error="Выберите вариант из списка" promptTitle="Тип клиента" prompt="Выберите один вариант" type="list">
-      <formula1>"Заказчик,Подрядчик,Сетевая компания,Проектный институт,Интегратор,Коммерческая организация,OEM"</formula1>
+      <formula1>"Холдинг,Заказчик,Подрядчик,Интегратор,Сетевая компания,OEM,Дистрибьютор,Проектный институт"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:L504" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Потенциал" error="Только целое число, без запятой: 5, а не 5,5" promptTitle="Потенциал" prompt="Сумма в млн ₽ в год, без запятой. Нет потенциала - оставьте пустым" type="whole" operator="between">
       <formula1>0</formula1>

</xml_diff>